<commit_message>
Corregir las hojas que la foto no dejaba leer con certeza.
El registro de ventas queda solo con los encabezados, porque las celdas de datos no se distinguen. En las demás hojas se ajustan la fórmula CONTARA, las cifras del dashboard y varias filas de estandarización.

Co-authored-by: sebsotoosolis-ui <sebsotoosolis-ui@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/documentos/Dashboard de ventas.xlsx
+++ b/documentos/Dashboard de ventas.xlsx
@@ -122,7 +122,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -158,11 +158,104 @@
         <color rgb="00E39B2B"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00E39B2B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00E39B2B"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00E39B2B"/>
+      </right>
+      <top style="medium">
+        <color rgb="00E39B2B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00E39B2B"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00E39B2B"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00E39B2B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00E39B2B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00E39B2B"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00E39B2B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00E39B2B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00E39B2B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00E39B2B"/>
+      </right>
+      <top style="medium">
+        <color rgb="00E39B2B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00E39B2B"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -240,6 +333,13 @@
     <xf numFmtId="1" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -318,7 +418,6 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -359,7 +458,7 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="1B3A4B"/>
+                <a:srgbClr val="1F4E4A"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -440,7 +539,6 @@
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
     <title>
       <tx>
@@ -478,7 +576,7 @@
             <idx val="0"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="1B3A4B"/>
+                <a:srgbClr val="1F4E4A"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -489,7 +587,7 @@
             <idx val="1"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="E39B2B"/>
+                <a:srgbClr val="E0A020"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -533,7 +631,7 @@
             <idx val="5"/>
             <spPr>
               <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:srgbClr val="2E75B6"/>
+                <a:srgbClr val="2E5090"/>
               </a:solidFill>
               <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
@@ -975,17 +1073,6 @@
           <t>DASHBOARD DE VENTAS</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
-      <c r="I1" s="2" t="n"/>
-      <c r="J1" s="2" t="n"/>
-      <c r="K1" s="2" t="n"/>
-      <c r="L1" s="2" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
@@ -993,17 +1080,6 @@
           <t>Resumen visual para el gerente — septiembre 2026</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
-      <c r="F2" s="4" t="n"/>
-      <c r="G2" s="4" t="n"/>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
-      <c r="J2" s="4" t="n"/>
-      <c r="K2" s="4" t="n"/>
-      <c r="L2" s="4" t="n"/>
     </row>
     <row r="3" ht="10" customHeight="1"/>
     <row r="4" ht="22" customHeight="1">
@@ -1012,66 +1088,66 @@
           <t>Ventas totales</t>
         </is>
       </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
+      <c r="B4" s="29" t="n"/>
+      <c r="C4" s="30" t="n"/>
       <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Cumplen meta</t>
         </is>
       </c>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
+      <c r="F4" s="29" t="n"/>
+      <c r="G4" s="30" t="n"/>
       <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Ventas destacadas</t>
         </is>
       </c>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="n"/>
+      <c r="I4" s="29" t="n"/>
+      <c r="J4" s="30" t="n"/>
       <c r="K4" s="5" t="inlineStr">
         <is>
           <t>A revisar</t>
         </is>
       </c>
-      <c r="L4" s="6" t="n"/>
+      <c r="L4" s="30" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="7">
         <f>KPIs!B2</f>
         <v/>
       </c>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
+      <c r="B5" s="31" t="n"/>
+      <c r="C5" s="32" t="n"/>
       <c r="E5" s="9">
         <f>KPIs!B3</f>
         <v/>
       </c>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
+      <c r="F5" s="31" t="n"/>
+      <c r="G5" s="32" t="n"/>
       <c r="H5" s="9">
         <f>KPIs!B4</f>
         <v/>
       </c>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
+      <c r="I5" s="31" t="n"/>
+      <c r="J5" s="32" t="n"/>
       <c r="K5" s="9">
         <f>KPIs!B5</f>
         <v/>
       </c>
-      <c r="L5" s="8" t="n"/>
+      <c r="L5" s="32" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
+      <c r="A6" s="33" t="n"/>
+      <c r="B6" s="34" t="n"/>
+      <c r="C6" s="35" t="n"/>
+      <c r="E6" s="33" t="n"/>
+      <c r="F6" s="34" t="n"/>
+      <c r="G6" s="35" t="n"/>
+      <c r="H6" s="33" t="n"/>
+      <c r="I6" s="34" t="n"/>
+      <c r="J6" s="35" t="n"/>
+      <c r="K6" s="33" t="n"/>
+      <c r="L6" s="35" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="10" t="inlineStr">
@@ -1277,7 +1353,7 @@
         </is>
       </c>
       <c r="B2" s="23" t="n">
-        <v>70500</v>
+        <v>73000</v>
       </c>
     </row>
     <row r="3">
@@ -1297,7 +1373,7 @@
         </is>
       </c>
       <c r="B4" s="23" t="n">
-        <v>87000</v>
+        <v>67000</v>
       </c>
     </row>
     <row r="5">
@@ -1317,7 +1393,7 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>74800</v>
+        <v>78800</v>
       </c>
     </row>
     <row r="7">
@@ -1347,7 +1423,7 @@
         </is>
       </c>
       <c r="B9" s="25" t="n">
-        <v>45200</v>
+        <v>44200</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -1369,7 +1445,7 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>305900</v>
+        <v>305500</v>
       </c>
     </row>
     <row r="14">
@@ -1379,7 +1455,7 @@
         </is>
       </c>
       <c r="B14" s="25" t="n">
-        <v>178200</v>
+        <v>178300</v>
       </c>
     </row>
     <row r="15">
@@ -1389,7 +1465,7 @@
         </is>
       </c>
       <c r="B15" s="23" t="n">
-        <v>87800</v>
+        <v>87200</v>
       </c>
     </row>
     <row r="16">

</xml_diff>